<commit_message>
Template approval in progress
</commit_message>
<xml_diff>
--- a/MessageTemplate_brief.xlsx
+++ b/MessageTemplate_brief.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8db45e9a3c2998f6/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MY REPO\Valcura\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{586CA3B4-6BF4-4E37-9F7F-7C124F63D5A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEE5BA65-6982-48CE-8C28-42A5D4035F6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A691CC11-0C54-47A6-93A5-F1D50936F339}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A691CC11-0C54-47A6-93A5-F1D50936F339}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -8194,12 +8194,30 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -8229,7 +8247,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -8240,13 +8258,40 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -8562,18 +8607,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9AB995C1-FA27-4AF9-9BC1-4E41583C278C}">
   <dimension ref="A1:H122"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="33.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="33.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="25" customWidth="1"/>
-    <col min="6" max="6" width="44.33203125" customWidth="1"/>
-    <col min="7" max="7" width="17.44140625" customWidth="1"/>
-    <col min="8" max="8" width="17.88671875" customWidth="1"/>
+    <col min="6" max="6" width="44.28515625" customWidth="1"/>
+    <col min="7" max="7" width="17.42578125" customWidth="1"/>
+    <col min="8" max="8" width="17.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -8599,7 +8644,7 @@
         <v>442</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="186" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" ht="180" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>2</v>
       </c>
@@ -8625,7 +8670,7 @@
         <v>443</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="212.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" ht="218.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>4</v>
       </c>
@@ -8651,215 +8696,215 @@
         <v>444</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="186" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="4" t="s">
+    <row r="4" spans="1:8" s="10" customFormat="1" ht="192.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="7" t="s">
         <v>245</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="8" t="s">
         <v>260</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="7" t="s">
         <v>261</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="F4" s="8" t="s">
         <v>317</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="G4" s="8" t="s">
         <v>438</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="H4" s="8" t="s">
         <v>443</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="186" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="4" t="s">
+    <row r="5" spans="1:8" s="10" customFormat="1" ht="180" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="7" t="s">
         <v>245</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="8" t="s">
         <v>260</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E5" s="7" t="s">
         <v>262</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="F5" s="9" t="s">
         <v>318</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="G5" s="8" t="s">
         <v>439</v>
       </c>
-      <c r="H5" s="2" t="s">
+      <c r="H5" s="8" t="s">
         <v>443</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="212.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="4" t="s">
+    <row r="6" spans="1:8" s="10" customFormat="1" ht="205.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="7" t="s">
         <v>246</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="8" t="s">
         <v>263</v>
       </c>
-      <c r="E6" s="5">
+      <c r="E6" s="14">
         <v>0</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="F6" s="9" t="s">
         <v>319</v>
       </c>
-      <c r="G6" s="2" t="s">
+      <c r="G6" s="8" t="s">
         <v>438</v>
       </c>
-      <c r="H6" s="2" t="s">
+      <c r="H6" s="8" t="s">
         <v>445</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="252" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="4" t="s">
+    <row r="7" spans="1:8" s="13" customFormat="1" ht="243.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="11" t="s">
         <v>246</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D7" s="12" t="s">
         <v>264</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="E7" s="11" t="s">
         <v>259</v>
       </c>
-      <c r="F7" s="6" t="s">
+      <c r="F7" s="15" t="s">
         <v>320</v>
       </c>
-      <c r="G7" s="2" t="s">
+      <c r="G7" s="12" t="s">
         <v>437</v>
       </c>
-      <c r="H7" s="2" t="s">
+      <c r="H7" s="12" t="s">
         <v>446</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="238.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="4" t="s">
+    <row r="8" spans="1:8" s="10" customFormat="1" ht="231" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="7" t="s">
         <v>246</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="8" t="s">
         <v>265</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="E8" s="7" t="s">
         <v>261</v>
       </c>
-      <c r="F8" s="6" t="s">
+      <c r="F8" s="9" t="s">
         <v>321</v>
       </c>
-      <c r="G8" s="2" t="s">
+      <c r="G8" s="8" t="s">
         <v>437</v>
       </c>
-      <c r="H8" s="2" t="s">
+      <c r="H8" s="8" t="s">
         <v>446</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="225.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="4" t="s">
+    <row r="9" spans="1:8" s="10" customFormat="1" ht="218.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="7" t="s">
         <v>246</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="D9" s="8" t="s">
         <v>266</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="E9" s="7" t="s">
         <v>262</v>
       </c>
-      <c r="F9" s="6" t="s">
+      <c r="F9" s="9" t="s">
         <v>322</v>
       </c>
-      <c r="G9" s="2" t="s">
+      <c r="G9" s="8" t="s">
         <v>439</v>
       </c>
-      <c r="H9" s="2" t="s">
+      <c r="H9" s="8" t="s">
         <v>446</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="331.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="4" t="s">
+    <row r="10" spans="1:8" s="13" customFormat="1" ht="218.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="11" t="s">
         <v>247</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D10" s="12" t="s">
         <v>267</v>
       </c>
-      <c r="E10" s="4" t="s">
+      <c r="E10" s="11" t="s">
         <v>268</v>
       </c>
-      <c r="F10" s="6" t="s">
+      <c r="F10" s="15" t="s">
         <v>323</v>
       </c>
-      <c r="G10" s="2" t="s">
+      <c r="G10" s="12" t="s">
         <v>438</v>
       </c>
-      <c r="H10" s="2" t="s">
+      <c r="H10" s="12" t="s">
         <v>447</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="225.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="4" t="s">
+    <row r="11" spans="1:8" s="10" customFormat="1" ht="180" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="7" t="s">
         <v>247</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="D11" s="8" t="s">
         <v>269</v>
       </c>
-      <c r="E11" s="4" t="s">
+      <c r="E11" s="7" t="s">
         <v>270</v>
       </c>
-      <c r="F11" s="2" t="s">
+      <c r="F11" s="8" t="s">
         <v>324</v>
       </c>
-      <c r="G11" s="2" t="s">
+      <c r="G11" s="8" t="s">
         <v>438</v>
       </c>
-      <c r="H11" s="2" t="s">
+      <c r="H11" s="8" t="s">
         <v>448</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="278.39999999999998" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" ht="192.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
         <v>22</v>
       </c>
@@ -8885,267 +8930,267 @@
         <v>449</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="199.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="4" t="s">
+    <row r="13" spans="1:8" s="10" customFormat="1" ht="192.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="7" t="s">
         <v>248</v>
       </c>
-      <c r="D13" s="2" t="s">
+      <c r="D13" s="8" t="s">
         <v>273</v>
       </c>
-      <c r="E13" s="4" t="s">
+      <c r="E13" s="7" t="s">
         <v>268</v>
       </c>
-      <c r="F13" s="6" t="s">
+      <c r="F13" s="9" t="s">
         <v>326</v>
       </c>
-      <c r="G13" s="2" t="s">
+      <c r="G13" s="8" t="s">
         <v>438</v>
       </c>
-      <c r="H13" s="2" t="s">
+      <c r="H13" s="8" t="s">
         <v>450</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="384" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="4" t="s">
+    <row r="14" spans="1:8" s="10" customFormat="1" ht="371.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="C14" s="7" t="s">
         <v>248</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="D14" s="8" t="s">
         <v>274</v>
       </c>
-      <c r="E14" s="4" t="s">
+      <c r="E14" s="7" t="s">
         <v>275</v>
       </c>
-      <c r="F14" s="6" t="s">
+      <c r="F14" s="9" t="s">
         <v>327</v>
       </c>
-      <c r="G14" s="2" t="s">
+      <c r="G14" s="8" t="s">
         <v>437</v>
       </c>
-      <c r="H14" s="2" t="s">
+      <c r="H14" s="8" t="s">
         <v>451</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="238.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="4" t="s">
+    <row r="15" spans="1:8" s="10" customFormat="1" ht="231" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C15" s="7" t="s">
         <v>249</v>
       </c>
-      <c r="D15" s="2" t="s">
+      <c r="D15" s="8" t="s">
         <v>276</v>
       </c>
-      <c r="E15" s="4" t="s">
+      <c r="E15" s="7" t="s">
         <v>277</v>
       </c>
-      <c r="F15" s="6" t="s">
+      <c r="F15" s="9" t="s">
         <v>328</v>
       </c>
-      <c r="G15" s="2" t="s">
+      <c r="G15" s="8" t="s">
         <v>437</v>
       </c>
-      <c r="H15" s="2" t="s">
+      <c r="H15" s="8" t="s">
         <v>452</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="304.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="4" t="s">
+    <row r="16" spans="1:8" s="10" customFormat="1" ht="294.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="C16" s="7" t="s">
         <v>249</v>
       </c>
-      <c r="D16" s="2" t="s">
+      <c r="D16" s="8" t="s">
         <v>278</v>
       </c>
-      <c r="E16" s="4" t="s">
+      <c r="E16" s="7" t="s">
         <v>279</v>
       </c>
-      <c r="F16" s="6" t="s">
+      <c r="F16" s="9" t="s">
         <v>329</v>
       </c>
-      <c r="G16" s="2" t="s">
+      <c r="G16" s="8" t="s">
         <v>439</v>
       </c>
-      <c r="H16" s="2" t="s">
+      <c r="H16" s="8" t="s">
         <v>453</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="291.60000000000002" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="4" t="s">
+    <row r="17" spans="1:8" s="10" customFormat="1" ht="282" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="C17" s="7" t="s">
         <v>249</v>
       </c>
-      <c r="D17" s="2" t="s">
+      <c r="D17" s="8" t="s">
         <v>280</v>
       </c>
-      <c r="E17" s="4" t="s">
+      <c r="E17" s="7" t="s">
         <v>281</v>
       </c>
-      <c r="F17" s="6" t="s">
+      <c r="F17" s="9" t="s">
         <v>330</v>
       </c>
-      <c r="G17" s="2" t="s">
+      <c r="G17" s="8" t="s">
         <v>437</v>
       </c>
-      <c r="H17" s="2" t="s">
+      <c r="H17" s="8" t="s">
         <v>453</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="265.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="4" t="s">
+    <row r="18" spans="1:8" s="10" customFormat="1" ht="256.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="B18" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="C18" s="7" t="s">
         <v>249</v>
       </c>
-      <c r="D18" s="2" t="s">
+      <c r="D18" s="8" t="s">
         <v>282</v>
       </c>
-      <c r="E18" s="4" t="s">
+      <c r="E18" s="7" t="s">
         <v>277</v>
       </c>
-      <c r="F18" s="6" t="s">
+      <c r="F18" s="9" t="s">
         <v>331</v>
       </c>
-      <c r="G18" s="2" t="s">
+      <c r="G18" s="8" t="s">
         <v>437</v>
       </c>
-      <c r="H18" s="2" t="s">
+      <c r="H18" s="8" t="s">
         <v>452</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="265.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="4" t="s">
+    <row r="19" spans="1:8" s="10" customFormat="1" ht="256.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="B19" s="4" t="s">
+      <c r="B19" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="C19" s="4" t="s">
+      <c r="C19" s="7" t="s">
         <v>249</v>
       </c>
-      <c r="D19" s="2" t="s">
+      <c r="D19" s="8" t="s">
         <v>278</v>
       </c>
-      <c r="E19" s="4" t="s">
+      <c r="E19" s="7" t="s">
         <v>279</v>
       </c>
-      <c r="F19" s="6" t="s">
+      <c r="F19" s="9" t="s">
         <v>332</v>
       </c>
-      <c r="G19" s="2" t="s">
+      <c r="G19" s="8" t="s">
         <v>439</v>
       </c>
-      <c r="H19" s="2" t="s">
+      <c r="H19" s="8" t="s">
         <v>452</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="278.39999999999998" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="4" t="s">
+    <row r="20" spans="1:8" s="10" customFormat="1" ht="269.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B20" s="4" t="s">
+      <c r="B20" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="C20" s="4" t="s">
+      <c r="C20" s="7" t="s">
         <v>249</v>
       </c>
-      <c r="D20" s="2" t="s">
+      <c r="D20" s="8" t="s">
         <v>280</v>
       </c>
-      <c r="E20" s="4" t="s">
+      <c r="E20" s="7" t="s">
         <v>281</v>
       </c>
-      <c r="F20" s="6" t="s">
+      <c r="F20" s="9" t="s">
         <v>333</v>
       </c>
-      <c r="G20" s="2" t="s">
+      <c r="G20" s="8" t="s">
         <v>437</v>
       </c>
-      <c r="H20" s="2" t="s">
+      <c r="H20" s="8" t="s">
         <v>452</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="304.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="4" t="s">
+    <row r="21" spans="1:8" s="10" customFormat="1" ht="294.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="B21" s="4" t="s">
+      <c r="B21" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="C21" s="4" t="s">
+      <c r="C21" s="7" t="s">
         <v>249</v>
       </c>
-      <c r="D21" s="2" t="s">
+      <c r="D21" s="8" t="s">
         <v>283</v>
       </c>
-      <c r="E21" s="4" t="s">
+      <c r="E21" s="7" t="s">
         <v>277</v>
       </c>
-      <c r="F21" s="6" t="s">
+      <c r="F21" s="9" t="s">
         <v>334</v>
       </c>
-      <c r="G21" s="2" t="s">
+      <c r="G21" s="8" t="s">
         <v>437</v>
       </c>
-      <c r="H21" s="2" t="s">
+      <c r="H21" s="8" t="s">
         <v>452</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="278.39999999999998" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="4" t="s">
+    <row r="22" spans="1:8" s="10" customFormat="1" ht="269.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="B22" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="C22" s="4" t="s">
+      <c r="C22" s="7" t="s">
         <v>249</v>
       </c>
-      <c r="D22" s="2" t="s">
+      <c r="D22" s="8" t="s">
         <v>278</v>
       </c>
-      <c r="E22" s="4" t="s">
+      <c r="E22" s="7" t="s">
         <v>279</v>
       </c>
-      <c r="F22" s="6" t="s">
+      <c r="F22" s="9" t="s">
         <v>335</v>
       </c>
-      <c r="G22" s="2" t="s">
+      <c r="G22" s="8" t="s">
         <v>439</v>
       </c>
-      <c r="H22" s="2" t="s">
+      <c r="H22" s="8" t="s">
         <v>452</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="278.39999999999998" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:8" ht="282" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
         <v>44</v>
       </c>
@@ -9171,7 +9216,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="225.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:8" ht="218.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
         <v>46</v>
       </c>
@@ -9197,7 +9242,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="278.39999999999998" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:8" ht="269.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="4" t="s">
         <v>48</v>
       </c>
@@ -9223,7 +9268,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="225.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:8" ht="231" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
         <v>50</v>
       </c>
@@ -9249,7 +9294,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="265.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:8" ht="269.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
         <v>52</v>
       </c>
@@ -9275,7 +9320,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="265.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:8" ht="256.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
         <v>54</v>
       </c>
@@ -9301,7 +9346,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="265.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:8" ht="256.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="4" t="s">
         <v>56</v>
       </c>
@@ -9327,7 +9372,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="252" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:8" ht="243.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="4" t="s">
         <v>58</v>
       </c>
@@ -9353,7 +9398,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="291.60000000000002" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:8" ht="282" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
         <v>60</v>
       </c>
@@ -9379,7 +9424,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="32" spans="1:8" ht="291.60000000000002" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:8" ht="282" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="4" t="s">
         <v>62</v>
       </c>
@@ -9405,7 +9450,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="278.39999999999998" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:8" ht="269.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="4" t="s">
         <v>64</v>
       </c>
@@ -9431,7 +9476,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="34" spans="1:8" ht="252" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:8" ht="256.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
         <v>66</v>
       </c>
@@ -9457,7 +9502,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="35" spans="1:8" ht="252" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:8" ht="243.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="4" t="s">
         <v>68</v>
       </c>
@@ -9483,7 +9528,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="36" spans="1:8" ht="212.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:8" ht="205.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="4" t="s">
         <v>70</v>
       </c>
@@ -9509,7 +9554,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="37" spans="1:8" ht="265.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:8" ht="256.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="4" t="s">
         <v>72</v>
       </c>
@@ -9535,7 +9580,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="38" spans="1:8" ht="291.60000000000002" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:8" ht="294.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="4" t="s">
         <v>74</v>
       </c>
@@ -9561,7 +9606,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="39" spans="1:8" ht="225.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:8" ht="218.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="4" t="s">
         <v>76</v>
       </c>
@@ -9587,7 +9632,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="40" spans="1:8" ht="252" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:8" ht="243.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="4" t="s">
         <v>78</v>
       </c>
@@ -9613,7 +9658,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="41" spans="1:8" ht="225.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:8" ht="218.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="4" t="s">
         <v>80</v>
       </c>
@@ -9639,7 +9684,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="42" spans="1:8" ht="265.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:8" ht="269.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="4" t="s">
         <v>82</v>
       </c>
@@ -9665,7 +9710,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="43" spans="1:8" ht="252" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:8" ht="243.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="4" t="s">
         <v>84</v>
       </c>
@@ -9691,7 +9736,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="44" spans="1:8" ht="278.39999999999998" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:8" ht="269.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="4" t="s">
         <v>86</v>
       </c>
@@ -9717,7 +9762,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="45" spans="1:8" ht="199.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:8" ht="205.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="4" t="s">
         <v>88</v>
       </c>
@@ -9743,7 +9788,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="46" spans="1:8" ht="278.39999999999998" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:8" ht="269.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="4" t="s">
         <v>90</v>
       </c>
@@ -9769,7 +9814,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="47" spans="1:8" ht="265.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:8" ht="256.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="4" t="s">
         <v>92</v>
       </c>
@@ -9795,7 +9840,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="48" spans="1:8" ht="252" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:8" ht="243.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="4" t="s">
         <v>94</v>
       </c>
@@ -9821,7 +9866,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="49" spans="1:8" ht="212.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:8" ht="218.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A49" s="4" t="s">
         <v>96</v>
       </c>
@@ -9847,33 +9892,33 @@
         <v>454</v>
       </c>
     </row>
-    <row r="50" spans="1:8" ht="238.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A50" s="4" t="s">
+    <row r="50" spans="1:8" s="19" customFormat="1" ht="231" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="16" t="s">
         <v>98</v>
       </c>
-      <c r="B50" s="4" t="s">
+      <c r="B50" s="16" t="s">
         <v>99</v>
       </c>
-      <c r="C50" s="4" t="s">
+      <c r="C50" s="16" t="s">
         <v>249</v>
       </c>
-      <c r="D50" s="2" t="s">
+      <c r="D50" s="17" t="s">
         <v>280</v>
       </c>
-      <c r="E50" s="4" t="s">
+      <c r="E50" s="16" t="s">
         <v>281</v>
       </c>
-      <c r="F50" s="6" t="s">
+      <c r="F50" s="18" t="s">
         <v>363</v>
       </c>
-      <c r="G50" s="2" t="s">
+      <c r="G50" s="17" t="s">
         <v>437</v>
       </c>
-      <c r="H50" s="2" t="s">
+      <c r="H50" s="17" t="s">
         <v>454</v>
       </c>
     </row>
-    <row r="51" spans="1:8" ht="212.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:8" ht="205.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A51" s="4" t="s">
         <v>100</v>
       </c>
@@ -9899,7 +9944,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="52" spans="1:8" ht="212.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:8" ht="205.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="4" t="s">
         <v>102</v>
       </c>
@@ -9925,7 +9970,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="53" spans="1:8" ht="238.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:8" ht="231" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="4" t="s">
         <v>104</v>
       </c>
@@ -9951,7 +9996,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="54" spans="1:8" ht="225.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:8" ht="218.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A54" s="4" t="s">
         <v>106</v>
       </c>
@@ -9977,7 +10022,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="55" spans="1:8" ht="238.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:8" ht="243.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A55" s="4" t="s">
         <v>108</v>
       </c>
@@ -10003,7 +10048,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="56" spans="1:8" ht="212.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:8" ht="218.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A56" s="4" t="s">
         <v>110</v>
       </c>
@@ -10029,7 +10074,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="57" spans="1:8" ht="225.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:8" ht="231" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A57" s="4" t="s">
         <v>112</v>
       </c>
@@ -10055,7 +10100,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="58" spans="1:8" ht="252" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:8" ht="243.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A58" s="4" t="s">
         <v>114</v>
       </c>
@@ -10081,7 +10126,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="59" spans="1:8" ht="265.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:8" ht="256.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A59" s="4" t="s">
         <v>116</v>
       </c>
@@ -10107,7 +10152,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="60" spans="1:8" ht="238.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:8" ht="231" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A60" s="4" t="s">
         <v>118</v>
       </c>
@@ -10133,7 +10178,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="61" spans="1:8" ht="278.39999999999998" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:8" ht="269.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A61" s="4" t="s">
         <v>120</v>
       </c>
@@ -10159,7 +10204,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="62" spans="1:8" ht="291.60000000000002" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:8" ht="282" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A62" s="4" t="s">
         <v>122</v>
       </c>
@@ -10185,7 +10230,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="63" spans="1:8" ht="238.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:8" ht="243.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A63" s="4" t="s">
         <v>124</v>
       </c>
@@ -10211,7 +10256,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="64" spans="1:8" ht="252" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:8" ht="243.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A64" s="4" t="s">
         <v>126</v>
       </c>
@@ -10237,7 +10282,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="65" spans="1:8" ht="238.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:8" ht="231" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A65" s="4" t="s">
         <v>128</v>
       </c>
@@ -10263,7 +10308,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="66" spans="1:8" ht="238.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:8" ht="231" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A66" s="4" t="s">
         <v>130</v>
       </c>
@@ -10289,7 +10334,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="67" spans="1:8" ht="199.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:8" ht="192.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A67" s="4" t="s">
         <v>132</v>
       </c>
@@ -10315,7 +10360,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="68" spans="1:8" ht="265.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:8" ht="256.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A68" s="4" t="s">
         <v>134</v>
       </c>
@@ -10341,7 +10386,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="69" spans="1:8" ht="252" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:8" ht="243.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A69" s="4" t="s">
         <v>136</v>
       </c>
@@ -10367,7 +10412,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="70" spans="1:8" ht="252" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:8" ht="243.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A70" s="4" t="s">
         <v>138</v>
       </c>
@@ -10393,7 +10438,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="71" spans="1:8" ht="225.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:8" ht="218.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A71" s="4" t="s">
         <v>140</v>
       </c>
@@ -10419,7 +10464,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="72" spans="1:8" ht="265.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:8" ht="256.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A72" s="4" t="s">
         <v>142</v>
       </c>
@@ -10445,7 +10490,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="73" spans="1:8" ht="265.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:8" ht="256.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A73" s="4" t="s">
         <v>144</v>
       </c>
@@ -10471,7 +10516,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="74" spans="1:8" ht="238.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:8" ht="231" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A74" s="4" t="s">
         <v>146</v>
       </c>
@@ -10497,7 +10542,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="75" spans="1:8" ht="238.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:8" ht="231" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A75" s="4" t="s">
         <v>148</v>
       </c>
@@ -10523,7 +10568,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="76" spans="1:8" ht="278.39999999999998" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:8" ht="269.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A76" s="4" t="s">
         <v>150</v>
       </c>
@@ -10549,7 +10594,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="77" spans="1:8" ht="225.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:8" ht="218.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A77" s="4" t="s">
         <v>152</v>
       </c>
@@ -10575,7 +10620,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="78" spans="1:8" ht="225.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:8" ht="231" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A78" s="4" t="s">
         <v>154</v>
       </c>
@@ -10601,7 +10646,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="79" spans="1:8" ht="238.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:8" ht="231" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A79" s="4" t="s">
         <v>156</v>
       </c>
@@ -10627,7 +10672,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="80" spans="1:8" ht="238.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:8" ht="243.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A80" s="4" t="s">
         <v>158</v>
       </c>
@@ -10653,7 +10698,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="81" spans="1:8" ht="225.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:8" ht="218.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A81" s="4" t="s">
         <v>160</v>
       </c>
@@ -10679,7 +10724,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="82" spans="1:8" ht="238.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:8" ht="231" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A82" s="4" t="s">
         <v>162</v>
       </c>
@@ -10705,7 +10750,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="83" spans="1:8" ht="265.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:8" ht="256.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A83" s="4" t="s">
         <v>164</v>
       </c>
@@ -10731,7 +10776,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="84" spans="1:8" ht="212.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:8" ht="205.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A84" s="4" t="s">
         <v>166</v>
       </c>
@@ -10757,7 +10802,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="85" spans="1:8" ht="212.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:8" ht="205.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A85" s="4" t="s">
         <v>168</v>
       </c>
@@ -10783,7 +10828,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="86" spans="1:8" ht="225.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:8" ht="218.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A86" s="4" t="s">
         <v>170</v>
       </c>
@@ -10809,7 +10854,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="87" spans="1:8" ht="278.39999999999998" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:8" ht="269.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A87" s="4" t="s">
         <v>172</v>
       </c>
@@ -10835,7 +10880,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="88" spans="1:8" ht="225.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:8" ht="218.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A88" s="4" t="s">
         <v>174</v>
       </c>
@@ -10861,7 +10906,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="89" spans="1:8" ht="238.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:8" ht="231" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A89" s="4" t="s">
         <v>176</v>
       </c>
@@ -10887,7 +10932,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="90" spans="1:8" ht="252" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:8" ht="256.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A90" s="4" t="s">
         <v>178</v>
       </c>
@@ -10913,7 +10958,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="91" spans="1:8" ht="252" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:8" ht="243.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A91" s="4" t="s">
         <v>180</v>
       </c>
@@ -10939,7 +10984,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="92" spans="1:8" ht="225.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:8" ht="218.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A92" s="4" t="s">
         <v>182</v>
       </c>
@@ -10965,7 +11010,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="93" spans="1:8" ht="265.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:8" ht="256.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A93" s="4" t="s">
         <v>184</v>
       </c>
@@ -10991,7 +11036,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="94" spans="1:8" ht="199.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:8" ht="192.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A94" s="4" t="s">
         <v>186</v>
       </c>
@@ -11017,7 +11062,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="95" spans="1:8" ht="225.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:8" ht="231" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A95" s="4" t="s">
         <v>188</v>
       </c>
@@ -11043,7 +11088,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="96" spans="1:8" ht="212.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:8" ht="205.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A96" s="4" t="s">
         <v>190</v>
       </c>
@@ -11069,7 +11114,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="97" spans="1:8" ht="225.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:8" ht="218.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A97" s="4" t="s">
         <v>192</v>
       </c>
@@ -11095,7 +11140,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="98" spans="1:8" ht="252" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:8" ht="243.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A98" s="4" t="s">
         <v>194</v>
       </c>
@@ -11121,7 +11166,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="99" spans="1:8" ht="212.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:8" ht="205.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A99" s="4" t="s">
         <v>196</v>
       </c>
@@ -11147,7 +11192,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="100" spans="1:8" ht="225.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:8" ht="218.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A100" s="4" t="s">
         <v>198</v>
       </c>
@@ -11173,7 +11218,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="101" spans="1:8" ht="172.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:8" ht="167.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A101" s="4" t="s">
         <v>200</v>
       </c>
@@ -11199,7 +11244,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="102" spans="1:8" ht="252" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:8" ht="243.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A102" s="4" t="s">
         <v>202</v>
       </c>
@@ -11225,7 +11270,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="103" spans="1:8" ht="252" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:8" ht="243.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A103" s="4" t="s">
         <v>204</v>
       </c>
@@ -11251,7 +11296,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="104" spans="1:8" ht="212.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:8" ht="231" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A104" s="4" t="s">
         <v>206</v>
       </c>
@@ -11277,7 +11322,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="105" spans="1:8" ht="265.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:8" ht="256.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A105" s="4" t="s">
         <v>208</v>
       </c>
@@ -11303,7 +11348,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="106" spans="1:8" ht="265.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:8" ht="256.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A106" s="4" t="s">
         <v>210</v>
       </c>
@@ -11329,7 +11374,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="107" spans="1:8" ht="265.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:8" ht="256.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A107" s="4" t="s">
         <v>212</v>
       </c>
@@ -11355,7 +11400,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="108" spans="1:8" ht="265.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:8" ht="256.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A108" s="4" t="s">
         <v>214</v>
       </c>
@@ -11381,7 +11426,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="109" spans="1:8" ht="278.39999999999998" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:8" ht="269.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A109" s="4" t="s">
         <v>216</v>
       </c>
@@ -11407,7 +11452,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="110" spans="1:8" ht="265.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:8" ht="269.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A110" s="4" t="s">
         <v>218</v>
       </c>
@@ -11433,7 +11478,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="111" spans="1:8" ht="304.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:8" ht="320.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A111" s="4" t="s">
         <v>220</v>
       </c>
@@ -11459,7 +11504,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="112" spans="1:8" ht="278.39999999999998" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:8" ht="269.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A112" s="4" t="s">
         <v>222</v>
       </c>
@@ -11485,7 +11530,7 @@
         <v>458</v>
       </c>
     </row>
-    <row r="113" spans="1:8" ht="238.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:8" ht="231" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A113" s="4" t="s">
         <v>224</v>
       </c>
@@ -11511,7 +11556,7 @@
         <v>458</v>
       </c>
     </row>
-    <row r="114" spans="1:8" ht="278.39999999999998" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:8" ht="269.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A114" s="4" t="s">
         <v>226</v>
       </c>
@@ -11537,7 +11582,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="115" spans="1:8" ht="344.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:8" ht="333" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A115" s="4" t="s">
         <v>228</v>
       </c>
@@ -11563,7 +11608,7 @@
         <v>459</v>
       </c>
     </row>
-    <row r="116" spans="1:8" ht="318" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:8" ht="307.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A116" s="4" t="s">
         <v>230</v>
       </c>
@@ -11589,7 +11634,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="117" spans="1:8" ht="291.60000000000002" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:8" ht="282" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A117" s="4" t="s">
         <v>232</v>
       </c>
@@ -11615,7 +11660,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="118" spans="1:8" ht="238.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:8" ht="231" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A118" s="4" t="s">
         <v>234</v>
       </c>
@@ -11641,7 +11686,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="119" spans="1:8" ht="291.60000000000002" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:8" ht="294.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A119" s="4" t="s">
         <v>236</v>
       </c>
@@ -11667,7 +11712,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="120" spans="1:8" ht="225.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:8" ht="231" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A120" s="4" t="s">
         <v>238</v>
       </c>
@@ -11693,7 +11738,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="121" spans="1:8" ht="278.39999999999998" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:8" ht="269.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A121" s="4" t="s">
         <v>240</v>
       </c>
@@ -11719,7 +11764,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="122" spans="1:8" ht="278.39999999999998" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:8" ht="269.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A122" s="4" t="s">
         <v>242</v>
       </c>

</xml_diff>